<commit_message>
Fase 160: ejemplos de la plantilla de Flujo de WhatsApp en el formato que lee el sistema (v1.58.1)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/server/plantillas/PLANTILLA_FLUJO_WHATSAPP.xlsx
+++ b/server/plantillas/PLANTILLA_FLUJO_WHATSAPP.xlsx
@@ -638,10 +638,10 @@
         <v>No</v>
       </c>
       <c r="C14" t="str">
-        <v>% atendidas en 10 s.</v>
-      </c>
-      <c r="D14">
-        <v>0.4</v>
+        <v>% atendidas en 10 s. Como porcentaje ("40 %" o celda con formato %).</v>
+      </c>
+      <c r="D14" t="str">
+        <v>40.00 %</v>
       </c>
       <c r="E14" t="str">
         <v/>
@@ -655,10 +655,10 @@
         <v>No</v>
       </c>
       <c r="C15" t="str">
-        <v>% atendidas en 20 s.</v>
-      </c>
-      <c r="D15">
-        <v>0.5</v>
+        <v>% atendidas en 20 s. Como porcentaje.</v>
+      </c>
+      <c r="D15" t="str">
+        <v>50.00 %</v>
       </c>
       <c r="E15" t="str">
         <v/>
@@ -672,10 +672,10 @@
         <v>No</v>
       </c>
       <c r="C16" t="str">
-        <v>% atendidas en 30 s.</v>
-      </c>
-      <c r="D16">
-        <v>0.6</v>
+        <v>% atendidas en 30 s. Como porcentaje.</v>
+      </c>
+      <c r="D16" t="str">
+        <v>60.00 %</v>
       </c>
       <c r="E16" t="str">
         <v/>
@@ -689,10 +689,10 @@
         <v>No</v>
       </c>
       <c r="C17" t="str">
-        <v>% atendidas en 5 min.</v>
-      </c>
-      <c r="D17">
-        <v>0.9</v>
+        <v>% atendidas en 5 min. Como porcentaje.</v>
+      </c>
+      <c r="D17" t="str">
+        <v>90.00 %</v>
       </c>
       <c r="E17" t="str">
         <v>SERVICE_LEVEL_300SEC, NIVEL DE SERVICIO 5 MIN</v>
@@ -706,7 +706,7 @@
         <v>No</v>
       </c>
       <c r="C18" t="str">
-        <v>Tiempo promedio de respuesta.</v>
+        <v>Tiempo promedio de respuesta, en segundos.</v>
       </c>
       <c r="D18">
         <v>60</v>
@@ -723,7 +723,7 @@
         <v>No</v>
       </c>
       <c r="C19" t="str">
-        <v>Tiempo promedio hasta el abandono.</v>
+        <v>Tiempo promedio hasta el abandono, en segundos.</v>
       </c>
       <c r="D19">
         <v>300</v>
@@ -740,10 +740,10 @@
         <v>No</v>
       </c>
       <c r="C20" t="str">
-        <v>Tiempo promedio de atención.</v>
-      </c>
-      <c r="D20">
-        <v>400</v>
+        <v>Tiempo promedio de atención, como hora de Excel (h:mm:ss). No en segundos: 400 se leería como 400 días y la carga se rechaza.</v>
+      </c>
+      <c r="D20" t="str">
+        <v>0:06:40</v>
       </c>
       <c r="E20" t="str">
         <v/>

</xml_diff>